<commit_message>
update: schema remove softdeletes
update: kuis view
update: layout
update: praktikan praktikum upload
</commit_message>
<xml_diff>
--- a/public/assets/template-upload-praktikum-praktikan.xlsx
+++ b/public/assets/template-upload-praktikum-praktikan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Template JJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746FEFF4-C7EC-4A0B-A01B-47F24D69695B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C28D524-81E9-4C9B-942A-2F7A46BC6F4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,10 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>NPM</t>
   </si>
@@ -39,17 +42,62 @@
     <t>NAMA</t>
   </si>
   <si>
+    <t>ASLAB_ID</t>
+  </si>
+  <si>
+    <t>DOSEN_ID</t>
+  </si>
+  <si>
+    <t>SESI_PRAKTIKUM_ID</t>
+  </si>
+  <si>
+    <t>9e74f48c-c45c-4457-92f3-7f42c073413b</t>
+  </si>
+  <si>
     <t>06.2024.1.01234</t>
   </si>
   <si>
+    <t>06.2024.1.01235</t>
+  </si>
+  <si>
+    <t>06.2024.1.01236</t>
+  </si>
+  <si>
+    <t>06.2024.1.01237</t>
+  </si>
+  <si>
     <t>Elaina Annisa Zahra</t>
+  </si>
+  <si>
+    <t>Ahmad Saiful Hamdan Jamaluddin</t>
+  </si>
+  <si>
+    <t>Rusli Firmansyah</t>
+  </si>
+  <si>
+    <t>Evie Frye</t>
+  </si>
+  <si>
+    <t>9ab862fa-5883-4113-9ac5-7f5a92d0e752</t>
+  </si>
+  <si>
+    <t>6e757ad5-b5b1-4715-bf45-7895f548fbe9</t>
+  </si>
+  <si>
+    <t>71aff859-0110-48cb-811d-4bd134a32fb6</t>
+  </si>
+  <si>
+    <t>ee798c3f-64b8-4aa6-b180-ff4f4308cbee</t>
+  </si>
+  <si>
+    <t>8f15e68d-aeb3-4030-be8a-d735267edd0f</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,6 +110,22 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -84,10 +148,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -369,30 +447,439 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="39.85546875" customWidth="1"/>
+    <col min="1" max="1" width="17" style="6" customWidth="1"/>
+    <col min="2" max="2" width="39.85546875" style="6" customWidth="1"/>
+    <col min="3" max="5" width="38.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3"/>
+      <c r="B30" s="3"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="3"/>
+      <c r="B35" s="3"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="3"/>
+      <c r="B42" s="3"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="3"/>
+      <c r="B46" s="3"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="3"/>
+      <c r="B54" s="3"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="3"/>
+      <c r="B56" s="3"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="3"/>
+      <c r="B58" s="3"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="3"/>
+      <c r="B60" s="3"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="3"/>
+      <c r="B62" s="3"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="3"/>
+      <c r="B63" s="3"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="3"/>
+      <c r="B64" s="3"/>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="3"/>
+      <c r="B65" s="3"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="3"/>
+      <c r="B66" s="3"/>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="3"/>
+      <c r="B67" s="3"/>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="3"/>
+      <c r="B68" s="3"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="3"/>
+      <c r="B69" s="3"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="3"/>
+      <c r="B70" s="3"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="3"/>
+      <c r="B71" s="3"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="3"/>
+      <c r="B72" s="3"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="3"/>
+      <c r="B73" s="3"/>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="3"/>
+      <c r="B74" s="3"/>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="3"/>
+      <c r="B75" s="3"/>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" s="3"/>
+      <c r="B77" s="3"/>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" s="3"/>
+      <c r="B78" s="3"/>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" s="3"/>
+      <c r="B79" s="3"/>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" s="3"/>
+      <c r="B80" s="3"/>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" s="3"/>
+      <c r="B81" s="3"/>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" s="3"/>
+      <c r="B82" s="3"/>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" s="3"/>
+      <c r="B83" s="3"/>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" s="3"/>
+      <c r="B84" s="3"/>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" s="3"/>
+      <c r="B85" s="3"/>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" s="3"/>
+      <c r="B86" s="3"/>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" s="3"/>
+      <c r="B87" s="3"/>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="3"/>
+      <c r="B88" s="3"/>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" s="3"/>
+      <c r="B89" s="3"/>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" s="3"/>
+      <c r="B90" s="3"/>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" s="3"/>
+      <c r="B91" s="3"/>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" s="3"/>
+      <c r="B92" s="3"/>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" s="3"/>
+      <c r="B93" s="3"/>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="5"/>
+      <c r="B94" s="5"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>